<commit_message>
Déploiment du protocole ospf pour le routage dynamique (réseau opérateur)
</commit_message>
<xml_diff>
--- a/docs/Resume_Table_addressage.xlsx
+++ b/docs/Resume_Table_addressage.xlsx
@@ -8,18 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\njlid\Desktop\cnam\cnam-24-25\RSX103\portfolio\Secure-Entrepise-Network-Architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E0F7F6-C387-42B1-A504-04A24250AFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFD6085-A3BC-4AD9-812E-027D0A082A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{95F63387-710A-4DE0-80EC-A390F828E8CA}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="15105" windowHeight="15585" firstSheet="2" activeTab="6" xr2:uid="{95F63387-710A-4DE0-80EC-A390F828E8CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil3" sheetId="3" r:id="rId1"/>
-    <sheet name="Q1- Plan d'adressage" sheetId="1" r:id="rId2"/>
+    <sheet name="Plan d'adressage sites" sheetId="1" r:id="rId2"/>
     <sheet name="Q2-Config_VLAN" sheetId="2" r:id="rId3"/>
     <sheet name="DHCP" sheetId="5" r:id="rId4"/>
     <sheet name="NAT" sheetId="6" r:id="rId5"/>
     <sheet name="ACL" sheetId="4" r:id="rId6"/>
-    <sheet name="Feuil1" sheetId="7" r:id="rId7"/>
+    <sheet name="Plan d'adressage R Op" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="533">
   <si>
     <t>Site</t>
   </si>
@@ -1303,84 +1303,6 @@
     <t>no access-list 100 permit ip any any</t>
   </si>
   <si>
-    <t>DHCP sur un serveur :</t>
-  </si>
-  <si>
-    <t>/etc/dhcp/dhcpd.conf</t>
-  </si>
-  <si>
-    <t>/etc/default/isc-dhcp-server</t>
-  </si>
-  <si>
-    <t>service isc-dhcp-server start</t>
-  </si>
-  <si>
-    <t>rm /var/run/dhcp.pid</t>
-  </si>
-  <si>
-    <t>/etc/init.d/networking restart (stop:start:..)</t>
-  </si>
-  <si>
-    <t>ss -anp</t>
-  </si>
-  <si>
-    <t>service isc-dhcp-relay start</t>
-  </si>
-  <si>
-    <t>DHCP sur Routeur</t>
-  </si>
-  <si>
-    <t>(config)#ip dhcp pool POOLlan1</t>
-  </si>
-  <si>
-    <t>(config)#network 192.168.1.0 255.255.255.0</t>
-  </si>
-  <si>
-    <t>(config)#default-router 192.168.1.1</t>
-  </si>
-  <si>
-    <t>(config)#no ip dhcp pool POOLlan1</t>
-  </si>
-  <si>
-    <t>(config)#ip dhcp excluded-address @ip_min @ip_max</t>
-  </si>
-  <si>
-    <t>exclure des adresses ip</t>
-  </si>
-  <si>
-    <t>show ip dhcp pool POOLlan1</t>
-  </si>
-  <si>
-    <t>show ip dhcp binding</t>
-  </si>
-  <si>
-    <t>www.cnam.fr est le nom internet complet</t>
-  </si>
-  <si>
-    <t>www est le nom de la machine</t>
-  </si>
-  <si>
-    <t>cnam.fr est le nom de domaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/etc/resolv.conf   si il est configuré en statique : </t>
-  </si>
-  <si>
-    <t>search mondomaine.fr</t>
-  </si>
-  <si>
-    <t>nameserver 192,168,50,90</t>
-  </si>
-  <si>
-    <t>nameserver 192,168,50,91</t>
-  </si>
-  <si>
-    <t xml:space="preserve">si le réseau est configuré de façon dynamique avec un dhcp </t>
-  </si>
-  <si>
-    <t>ou network-manager alors ce fichier sera modifié mis à jour autom</t>
-  </si>
-  <si>
     <r>
       <t>123.1</t>
     </r>
@@ -2006,12 +1928,447 @@
   <si>
     <t>ip access-group 102 out</t>
   </si>
+  <si>
+    <t>Découpage d'adressage</t>
+  </si>
+  <si>
+    <t>Lien</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IP réseau</t>
+  </si>
+  <si>
+    <t>IP1 -- IP2</t>
+  </si>
+  <si>
+    <t>Interfaces</t>
+  </si>
+  <si>
+    <t>R1 -- RO11 (A1)</t>
+  </si>
+  <si>
+    <t>R2 -- RO21 (B1)</t>
+  </si>
+  <si>
+    <t>RF1 -- RO31 (intra)</t>
+  </si>
+  <si>
+    <t>RF2 -- RO32 (public)</t>
+  </si>
+  <si>
+    <t>RO11 -- RO2</t>
+  </si>
+  <si>
+    <t>RO21 -- RO3</t>
+  </si>
+  <si>
+    <t>RO31 -- RO4</t>
+  </si>
+  <si>
+    <t>RO2 -- RO4</t>
+  </si>
+  <si>
+    <t>RO3 -- RO4</t>
+  </si>
+  <si>
+    <t>RO2 -- RO1</t>
+  </si>
+  <si>
+    <t>RO3 -- RO1</t>
+  </si>
+  <si>
+    <t>RO4 -- RO1</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>163.173.18.254/31</t>
+  </si>
+  <si>
+    <t>163.173.19.222/31</t>
+  </si>
+  <si>
+    <t>12.0.0.0/30</t>
+  </si>
+  <si>
+    <t>12.0.0.4/30</t>
+  </si>
+  <si>
+    <t>12.0.0.8/30</t>
+  </si>
+  <si>
+    <t>12.0.0.12/30</t>
+  </si>
+  <si>
+    <t>12.0.0.16/30</t>
+  </si>
+  <si>
+    <t>12.0.0.20/30</t>
+  </si>
+  <si>
+    <t>12.0.0.24/30</t>
+  </si>
+  <si>
+    <t>12.0.0.28/30</t>
+  </si>
+  <si>
+    <t>12.0.0.0</t>
+  </si>
+  <si>
+    <t>12.0.0.4</t>
+  </si>
+  <si>
+    <t>12.0.0.8</t>
+  </si>
+  <si>
+    <t>12.0.0.12</t>
+  </si>
+  <si>
+    <t>12.0.0.16</t>
+  </si>
+  <si>
+    <t>12.0.0.20</t>
+  </si>
+  <si>
+    <t>12.0.0.24</t>
+  </si>
+  <si>
+    <t>12.0.0.28</t>
+  </si>
+  <si>
+    <t>12.0.0.3</t>
+  </si>
+  <si>
+    <t>12.0.0.7</t>
+  </si>
+  <si>
+    <t>12.0.0.11</t>
+  </si>
+  <si>
+    <t>12.0.0.15</t>
+  </si>
+  <si>
+    <t>12.0.0.19</t>
+  </si>
+  <si>
+    <t>12.0.0.23</t>
+  </si>
+  <si>
+    <t>12.0.0.27</t>
+  </si>
+  <si>
+    <t>12.0.0.31</t>
+  </si>
+  <si>
+    <t>12.0.0.1 -- 12.0.0.2</t>
+  </si>
+  <si>
+    <t>12.0.0.5 -- 12.0.0.6</t>
+  </si>
+  <si>
+    <t>12.0.0.9 -- 12.0.0.10</t>
+  </si>
+  <si>
+    <t>12.0.0.13 -- 12.0.0.14</t>
+  </si>
+  <si>
+    <t>12.0.0.17 -- 12.0.0.18</t>
+  </si>
+  <si>
+    <t>12.0.0.21 -- 12.0.0.22</t>
+  </si>
+  <si>
+    <t>12.0.0.25 -- 12.0.0.26</t>
+  </si>
+  <si>
+    <t>12.0.0.29 -- 12.0.0.30</t>
+  </si>
+  <si>
+    <t>123.1.1.176 -- 123.1.1.177</t>
+  </si>
+  <si>
+    <t>123.2.2.168 -- 123.2.2.169</t>
+  </si>
+  <si>
+    <t>163.173.18.254 -- 163.173.18.255</t>
+  </si>
+  <si>
+    <t>163.173.19.222 -- 163.173.19.223</t>
+  </si>
+  <si>
+    <t>f0/0 -- f0/0</t>
+  </si>
+  <si>
+    <t>e1/0 -- e1/1</t>
+  </si>
+  <si>
+    <t>e1/0 -- e1/0</t>
+  </si>
+  <si>
+    <t>e1/3 -- e1/3</t>
+  </si>
+  <si>
+    <t>e1/1 -- e1/1</t>
+  </si>
+  <si>
+    <t>e1/2 -- e1/2</t>
+  </si>
+  <si>
+    <t>Sous-réseau/masque</t>
+  </si>
+  <si>
+    <t>Configuration des interfaces routeurs</t>
+  </si>
+  <si>
+    <t>Routeur</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface f0/0 </t>
+  </si>
+  <si>
+    <t>ip address 123.1.1.176 255.255.255.254</t>
+  </si>
+  <si>
+    <t>no shutdown</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>ip address 123.2.2.176 255.255.255.254</t>
+  </si>
+  <si>
+    <t>RO11</t>
+  </si>
+  <si>
+    <t>ip address 123.2.2.177 255.255.255.254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface e1/0 </t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.1 255.255.255.252</t>
+  </si>
+  <si>
+    <t>RO21</t>
+  </si>
+  <si>
+    <t>ip address 123.2.2.169 255.255.255.254</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.5 255.255.255.252</t>
+  </si>
+  <si>
+    <t>RO31</t>
+  </si>
+  <si>
+    <t>ip address 163.173.19.223 255.255.255.254</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.9 255.255.255.252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface e1/1 </t>
+  </si>
+  <si>
+    <t>ip address 163.173.19.225 255.255.255.254</t>
+  </si>
+  <si>
+    <t>RO1</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.22 255.255.255.252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface e1/2 </t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.29 255.255.255.252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface e1/3 </t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.26 255.255.255.252</t>
+  </si>
+  <si>
+    <t>RO2</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.2 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.21 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.13 255.255.255.252</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RO3 </t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.6 255.255.255.252</t>
+  </si>
+  <si>
+    <t>interface e1/1</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.17 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.25 255.255.255.252</t>
+  </si>
+  <si>
+    <t>RO4</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.10 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.18 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.30 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip address 12.0.0.14 255.255.255.252</t>
+  </si>
+  <si>
+    <t>Attribution d'adresse IP aux interfaces</t>
+  </si>
+  <si>
+    <t>Configuration route dynamique : OSPF</t>
+  </si>
+  <si>
+    <t>#Configure terminal</t>
+  </si>
+  <si>
+    <t>#router ospf 1</t>
+  </si>
+  <si>
+    <t>#network 12.0.0.0  0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t>#end</t>
+  </si>
+  <si>
+    <t>#router-id 11.11.11.11</t>
+  </si>
+  <si>
+    <t>#router-id 21.21.21.21</t>
+  </si>
+  <si>
+    <t>#network 12.0.0.4  0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t>#router-id 31.31.31.31</t>
+  </si>
+  <si>
+    <t>#network 12.0.0.8  0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># configure terminal</t>
+  </si>
+  <si>
+    <t># router ospf 1</t>
+  </si>
+  <si>
+    <t># router-id 1.1.1.1</t>
+  </si>
+  <si>
+    <t># network 12.0.0.20 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># network 12.0.0.28 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># network 12.0.0.24 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># end</t>
+  </si>
+  <si>
+    <t># router-id 2.2.2.2</t>
+  </si>
+  <si>
+    <t># network 12.0.0.0 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># network 12.0.0.12 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># router-id 3.3.3.3</t>
+  </si>
+  <si>
+    <t># network 12.0.0.4 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># network 12.0.0.16 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t># router-id 4.4.4.4</t>
+  </si>
+  <si>
+    <t># network 12.0.0.8 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t>#configuration terminal</t>
+  </si>
+  <si>
+    <t>#ip route 123.1.1.160 255.255.255.240 123.1.1.176</t>
+  </si>
+  <si>
+    <t>#Redistribute static subnets</t>
+  </si>
+  <si>
+    <t>#passive-interface f0/0</t>
+  </si>
+  <si>
+    <t>#network 123.1.1.176 0.0.0.1 area 0</t>
+  </si>
+  <si>
+    <t>#ip route 163.173.19.224 255.255.255.240 163.173.19.222</t>
+  </si>
+  <si>
+    <t>#network 163.173.19.222 0.0.0.1 area 0</t>
+  </si>
+  <si>
+    <t>#ip route 123.2.2.160 255.255.255.240 123.2.2.168</t>
+  </si>
+  <si>
+    <t>#network 123.2.2.168 0.0.0.1 area 0</t>
+  </si>
+  <si>
+    <t>ip route 0.0.0.0 0.0.0.0 123.1.1.177</t>
+  </si>
+  <si>
+    <t>ip route 0.0.0.0 0.0.0.0 123.2.2.169</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Route statique-route par défaut vers l'opérateur-interface passive</t>
+  </si>
+  <si>
+    <t>ip route 0.0.0.0 0.0.0.0 163.173.19.223</t>
+  </si>
+  <si>
+    <t>ip address 192.168.3.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 163.173.19.225 255.255.255.248</t>
+  </si>
+  <si>
+    <t>#  network 12.0.0.12 0.0.0.3 area 0</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2195,8 +2552,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2264,8 +2629,44 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -2336,8 +2737,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="10">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
@@ -2348,8 +2782,10 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2432,8 +2868,33 @@
     <xf numFmtId="0" fontId="21" fillId="7" borderId="4" xfId="3"/>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="4" xfId="2"/>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="7" xfId="10"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="6" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="11" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" xfId="10" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" xfId="10" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="8" xfId="10" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" xfId="10" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="10">
+  <cellStyles count="12">
+    <cellStyle name="20 % - Accent1" xfId="11" builtinId="30"/>
     <cellStyle name="20 % - Accent2" xfId="8" builtinId="34"/>
     <cellStyle name="20 % - Accent6" xfId="9" builtinId="50"/>
     <cellStyle name="40 % - Accent1" xfId="6" builtinId="31"/>
@@ -2444,6 +2905,7 @@
     <cellStyle name="Entrée" xfId="2" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Satisfaisant" xfId="1" builtinId="26"/>
+    <cellStyle name="Sortie" xfId="10" builtinId="21"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -2974,7 +3436,7 @@
   <sheetData>
     <row r="2" spans="3:14">
       <c r="C2" t="s">
-        <v>306</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="3:14">
@@ -3131,13 +3593,13 @@
         <v>16</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>308</v>
+        <v>282</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>301</v>
+        <v>275</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>300</v>
+        <v>274</v>
       </c>
       <c r="I8" s="2">
         <v>16</v>
@@ -3146,16 +3608,16 @@
         <v>14</v>
       </c>
       <c r="K8" t="s">
-        <v>299</v>
+        <v>273</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>58</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>297</v>
+        <v>271</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>304</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="3:14">
@@ -3277,10 +3739,10 @@
         <v>38</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>309</v>
+        <v>283</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>302</v>
+        <v>276</v>
       </c>
       <c r="I12" s="29">
         <v>8</v>
@@ -3289,16 +3751,16 @@
         <v>6</v>
       </c>
       <c r="K12" t="s">
-        <v>298</v>
+        <v>272</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>56</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>305</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="3:14">
@@ -3457,7 +3919,7 @@
     </row>
     <row r="23" spans="2:11">
       <c r="C23" t="s">
-        <v>307</v>
+        <v>281</v>
       </c>
       <c r="K23" s="12"/>
     </row>
@@ -3469,7 +3931,7 @@
         <v>76</v>
       </c>
       <c r="F25" t="s">
-        <v>317</v>
+        <v>291</v>
       </c>
       <c r="G25" t="s">
         <v>91</v>
@@ -3500,7 +3962,7 @@
         <v>80</v>
       </c>
       <c r="F27" t="s">
-        <v>310</v>
+        <v>284</v>
       </c>
       <c r="G27" t="s">
         <v>103</v>
@@ -3514,7 +3976,7 @@
         <v>80</v>
       </c>
       <c r="F28" t="s">
-        <v>311</v>
+        <v>285</v>
       </c>
       <c r="G28" t="s">
         <v>97</v>
@@ -3528,7 +3990,7 @@
         <v>80</v>
       </c>
       <c r="F29" t="s">
-        <v>312</v>
+        <v>286</v>
       </c>
       <c r="G29" t="s">
         <v>104</v>
@@ -3542,7 +4004,7 @@
         <v>80</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>324</v>
+        <v>298</v>
       </c>
       <c r="G30" s="11" t="s">
         <v>105</v>
@@ -3573,7 +4035,7 @@
         <v>80</v>
       </c>
       <c r="F32" t="s">
-        <v>313</v>
+        <v>287</v>
       </c>
       <c r="G32" t="s">
         <v>218</v>
@@ -3587,7 +4049,7 @@
         <v>80</v>
       </c>
       <c r="F33" t="s">
-        <v>314</v>
+        <v>288</v>
       </c>
       <c r="G33" t="s">
         <v>219</v>
@@ -3601,7 +4063,7 @@
         <v>80</v>
       </c>
       <c r="F34" t="s">
-        <v>315</v>
+        <v>289</v>
       </c>
       <c r="G34" t="s">
         <v>220</v>
@@ -3615,7 +4077,7 @@
         <v>80</v>
       </c>
       <c r="F35" t="s">
-        <v>316</v>
+        <v>290</v>
       </c>
       <c r="G35" t="s">
         <v>221</v>
@@ -3660,7 +4122,7 @@
         <v>80</v>
       </c>
       <c r="F38" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
       <c r="G38" t="s">
         <v>106</v>
@@ -3702,7 +4164,7 @@
         <v>80</v>
       </c>
       <c r="F41" t="s">
-        <v>319</v>
+        <v>293</v>
       </c>
       <c r="G41" t="s">
         <v>109</v>
@@ -3984,7 +4446,7 @@
     <row r="13" spans="3:11">
       <c r="E13" s="2"/>
       <c r="F13" t="s">
-        <v>320</v>
+        <v>294</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>75</v>
@@ -4069,21 +4531,21 @@
     </row>
     <row r="24" spans="1:10">
       <c r="C24" s="10" t="s">
-        <v>345</v>
+        <v>319</v>
       </c>
       <c r="D24" s="10"/>
     </row>
     <row r="25" spans="1:10" ht="24">
       <c r="D25" s="25" t="s">
-        <v>343</v>
+        <v>317</v>
       </c>
       <c r="H25" s="25" t="s">
-        <v>346</v>
+        <v>320</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="D27" s="32" t="s">
-        <v>344</v>
+        <v>318</v>
       </c>
       <c r="E27" s="32" t="s">
         <v>251</v>
@@ -4093,7 +4555,7 @@
       </c>
       <c r="G27" s="26"/>
       <c r="H27" s="32" t="s">
-        <v>349</v>
+        <v>323</v>
       </c>
       <c r="I27" s="32" t="s">
         <v>251</v>
@@ -4138,7 +4600,7 @@
         <v>256</v>
       </c>
       <c r="I29" s="28" t="s">
-        <v>347</v>
+        <v>321</v>
       </c>
       <c r="J29" s="27" t="s">
         <v>45</v>
@@ -4160,7 +4622,7 @@
         <v>257</v>
       </c>
       <c r="I30" s="28" t="s">
-        <v>348</v>
+        <v>322</v>
       </c>
       <c r="J30" s="27" t="s">
         <v>47</v>
@@ -4254,7 +4716,7 @@
         <v>189</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>321</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="2:13">
@@ -4580,10 +5042,10 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="35" t="s">
-        <v>352</v>
+        <v>326</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>355</v>
+        <v>329</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>243</v>
@@ -4596,13 +5058,13 @@
         <v>244</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>322</v>
+        <v>296</v>
       </c>
       <c r="F2" s="30" t="s">
         <v>245</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H2" s="30" t="s">
         <v>246</v>
@@ -4614,13 +5076,13 @@
       </c>
       <c r="B3" s="38"/>
       <c r="C3" s="31" t="s">
-        <v>328</v>
+        <v>302</v>
       </c>
       <c r="D3" t="s">
         <v>247</v>
       </c>
       <c r="E3" t="s">
-        <v>323</v>
+        <v>297</v>
       </c>
       <c r="F3" t="s">
         <v>42</v>
@@ -4637,13 +5099,13 @@
         <v>226</v>
       </c>
       <c r="B4" s="40" t="s">
-        <v>356</v>
+        <v>330</v>
       </c>
       <c r="D4" t="s">
-        <v>330</v>
+        <v>304</v>
       </c>
       <c r="E4" t="s">
-        <v>325</v>
+        <v>299</v>
       </c>
       <c r="F4" t="s">
         <v>263</v>
@@ -4658,13 +5120,13 @@
     <row r="5" spans="1:8">
       <c r="A5" s="33"/>
       <c r="B5" s="38" t="s">
-        <v>357</v>
+        <v>331</v>
       </c>
       <c r="D5" t="s">
-        <v>331</v>
+        <v>305</v>
       </c>
       <c r="E5" t="s">
-        <v>326</v>
+        <v>300</v>
       </c>
       <c r="F5" t="s">
         <v>45</v>
@@ -4683,19 +5145,19 @@
     <row r="7" spans="1:8">
       <c r="A7" s="33"/>
       <c r="B7" s="40" t="s">
-        <v>358</v>
+        <v>332</v>
       </c>
       <c r="D7" s="30" t="s">
         <v>244</v>
       </c>
       <c r="E7" s="30" t="s">
-        <v>322</v>
+        <v>296</v>
       </c>
       <c r="F7" s="30" t="s">
         <v>245</v>
       </c>
       <c r="G7" s="30" t="s">
-        <v>327</v>
+        <v>301</v>
       </c>
       <c r="H7" s="30" t="s">
         <v>246</v>
@@ -4706,25 +5168,25 @@
         <v>227</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>359</v>
+        <v>333</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>329</v>
+        <v>303</v>
       </c>
       <c r="D8" t="s">
         <v>247</v>
       </c>
       <c r="E8" t="s">
-        <v>334</v>
+        <v>308</v>
       </c>
       <c r="F8" t="s">
         <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>336</v>
+        <v>310</v>
       </c>
       <c r="H8" t="s">
-        <v>335</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -4733,19 +5195,19 @@
       </c>
       <c r="B9" s="38"/>
       <c r="D9" t="s">
-        <v>332</v>
+        <v>306</v>
       </c>
       <c r="E9" t="s">
-        <v>337</v>
+        <v>311</v>
       </c>
       <c r="F9" t="s">
         <v>263</v>
       </c>
       <c r="G9" t="s">
-        <v>338</v>
+        <v>312</v>
       </c>
       <c r="H9" t="s">
-        <v>341</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -4753,22 +5215,22 @@
         <v>231</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>360</v>
+        <v>334</v>
       </c>
       <c r="D10" t="s">
-        <v>333</v>
+        <v>307</v>
       </c>
       <c r="E10" t="s">
-        <v>339</v>
+        <v>313</v>
       </c>
       <c r="F10" t="s">
         <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>340</v>
+        <v>314</v>
       </c>
       <c r="H10" t="s">
-        <v>342</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -4776,7 +5238,7 @@
         <v>172</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>361</v>
+        <v>335</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -4788,7 +5250,7 @@
         <v>230</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>365</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="24">
@@ -4799,7 +5261,7 @@
         <v>162</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>350</v>
+        <v>324</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4807,14 +5269,14 @@
         <v>172</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>362</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="33"/>
       <c r="B16" s="38"/>
       <c r="D16" s="32" t="s">
-        <v>351</v>
+        <v>325</v>
       </c>
       <c r="E16" s="32" t="s">
         <v>253</v>
@@ -4823,7 +5285,7 @@
     <row r="17" spans="1:5">
       <c r="A17" s="33"/>
       <c r="B17" s="38" t="s">
-        <v>363</v>
+        <v>337</v>
       </c>
       <c r="D17" s="27" t="s">
         <v>254</v>
@@ -4835,7 +5297,7 @@
     <row r="18" spans="1:5">
       <c r="A18" s="33"/>
       <c r="B18" s="38" t="s">
-        <v>364</v>
+        <v>338</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>256</v>
@@ -4846,7 +5308,7 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="37" t="s">
-        <v>353</v>
+        <v>327</v>
       </c>
       <c r="B19" s="38"/>
       <c r="D19" s="27" t="s">
@@ -4887,7 +5349,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="37" t="s">
-        <v>354</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -4928,10 +5390,10 @@
   <sheetData>
     <row r="4" spans="2:20">
       <c r="E4" s="9" t="s">
-        <v>384</v>
+        <v>358</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>405</v>
+        <v>379</v>
       </c>
       <c r="T4" t="s">
         <v>156</v>
@@ -4944,10 +5406,10 @@
     </row>
     <row r="6" spans="2:20">
       <c r="B6" s="36" t="s">
-        <v>367</v>
+        <v>341</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>368</v>
+        <v>342</v>
       </c>
       <c r="D6" s="36" t="s">
         <v>147</v>
@@ -4956,19 +5418,19 @@
         <v>91</v>
       </c>
       <c r="G6" s="43" t="s">
-        <v>389</v>
+        <v>363</v>
       </c>
       <c r="H6" s="43" t="s">
-        <v>385</v>
+        <v>359</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>386</v>
+        <v>360</v>
       </c>
       <c r="J6" s="43" t="s">
-        <v>387</v>
+        <v>361</v>
       </c>
       <c r="K6" s="47" t="s">
-        <v>406</v>
+        <v>380</v>
       </c>
       <c r="M6" t="s">
         <v>149</v>
@@ -4982,22 +5444,22 @@
         <v>65</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E7" s="42" t="s">
-        <v>371</v>
+        <v>345</v>
       </c>
       <c r="G7" s="44">
         <v>100</v>
       </c>
       <c r="H7" s="45" t="s">
-        <v>366</v>
+        <v>340</v>
       </c>
       <c r="I7" s="45" t="s">
-        <v>398</v>
+        <v>372</v>
       </c>
       <c r="J7" s="45" t="s">
-        <v>388</v>
+        <v>362</v>
       </c>
       <c r="K7" s="46"/>
     </row>
@@ -5009,21 +5471,21 @@
         <v>63</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E8" s="42" t="s">
-        <v>372</v>
+        <v>346</v>
       </c>
       <c r="G8" s="45"/>
       <c r="H8" s="45" t="s">
-        <v>399</v>
+        <v>373</v>
       </c>
       <c r="I8" s="45" t="s">
-        <v>400</v>
+        <v>374</v>
       </c>
       <c r="J8" s="45"/>
       <c r="K8" s="46" t="s">
-        <v>407</v>
+        <v>381</v>
       </c>
       <c r="M8" t="s">
         <v>157</v>
@@ -5036,13 +5498,13 @@
       <c r="E9" s="42"/>
       <c r="G9" s="45"/>
       <c r="H9" s="45" t="s">
-        <v>390</v>
+        <v>364</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>390</v>
+        <v>364</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>391</v>
+        <v>365</v>
       </c>
       <c r="K9" s="46" t="s">
         <v>234</v>
@@ -5059,10 +5521,10 @@
         <v>66</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E10" s="42" t="s">
-        <v>380</v>
+        <v>354</v>
       </c>
       <c r="G10" s="45"/>
       <c r="H10" s="45"/>
@@ -5078,25 +5540,25 @@
         <v>67</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E11" s="42" t="s">
-        <v>382</v>
+        <v>356</v>
       </c>
       <c r="G11" s="44">
         <v>101</v>
       </c>
       <c r="H11" s="45" t="s">
-        <v>401</v>
+        <v>375</v>
       </c>
       <c r="I11" s="45" t="s">
-        <v>402</v>
+        <v>376</v>
       </c>
       <c r="J11" s="45" t="s">
-        <v>393</v>
+        <v>367</v>
       </c>
       <c r="K11" s="46" t="s">
-        <v>408</v>
+        <v>382</v>
       </c>
       <c r="M11" t="s">
         <v>223</v>
@@ -5110,17 +5572,17 @@
         <v>66</v>
       </c>
       <c r="D12" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E12" s="42" t="s">
-        <v>381</v>
+        <v>355</v>
       </c>
       <c r="G12" s="45"/>
       <c r="H12" s="45" t="s">
-        <v>403</v>
+        <v>377</v>
       </c>
       <c r="I12" s="45" t="s">
-        <v>404</v>
+        <v>378</v>
       </c>
       <c r="J12" s="45"/>
       <c r="K12" s="46" t="s">
@@ -5138,17 +5600,17 @@
         <v>67</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>383</v>
+        <v>357</v>
       </c>
       <c r="G13" s="45"/>
       <c r="H13" s="45" t="s">
-        <v>392</v>
+        <v>366</v>
       </c>
       <c r="I13" s="45" t="s">
-        <v>392</v>
+        <v>366</v>
       </c>
       <c r="J13" s="45"/>
       <c r="K13" s="46"/>
@@ -5166,7 +5628,7 @@
       <c r="I14" s="45"/>
       <c r="J14" s="45"/>
       <c r="K14" s="46" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
     </row>
     <row r="15" spans="2:20" ht="16.5" thickTop="1" thickBot="1">
@@ -5177,25 +5639,25 @@
         <v>67</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E15" s="42" t="s">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="G15" s="44">
         <v>102</v>
       </c>
       <c r="H15" s="45" t="s">
-        <v>394</v>
+        <v>368</v>
       </c>
       <c r="I15" s="45" t="s">
-        <v>396</v>
+        <v>370</v>
       </c>
       <c r="J15" s="45" t="s">
-        <v>397</v>
+        <v>371</v>
       </c>
       <c r="K15" s="46" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" spans="2:20" ht="16.5" thickTop="1" thickBot="1">
@@ -5206,17 +5668,17 @@
         <v>66</v>
       </c>
       <c r="D16" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E16" s="42" t="s">
-        <v>374</v>
+        <v>348</v>
       </c>
       <c r="G16" s="45"/>
       <c r="H16" s="45" t="s">
-        <v>395</v>
+        <v>369</v>
       </c>
       <c r="I16" s="45" t="s">
-        <v>395</v>
+        <v>369</v>
       </c>
       <c r="J16" s="45"/>
       <c r="K16" s="46"/>
@@ -5234,7 +5696,7 @@
       <c r="I17" s="45"/>
       <c r="J17" s="45"/>
       <c r="K17" s="46" t="s">
-        <v>411</v>
+        <v>385</v>
       </c>
       <c r="M17" t="s">
         <v>161</v>
@@ -5248,13 +5710,13 @@
         <v>63</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E18" s="42" t="s">
-        <v>375</v>
+        <v>349</v>
       </c>
       <c r="K18" s="46" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="M18" t="s">
         <v>162</v>
@@ -5268,10 +5730,10 @@
         <v>65</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E19" s="42" t="s">
-        <v>376</v>
+        <v>350</v>
       </c>
       <c r="M19" t="s">
         <v>163</v>
@@ -5285,11 +5747,11 @@
         <v>66</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E20" s="42"/>
       <c r="K20" s="46" t="s">
-        <v>412</v>
+        <v>386</v>
       </c>
     </row>
     <row r="21" spans="2:14" ht="16.5" thickTop="1" thickBot="1">
@@ -5300,13 +5762,13 @@
         <v>67</v>
       </c>
       <c r="D21" s="42" t="s">
-        <v>369</v>
+        <v>343</v>
       </c>
       <c r="E21" s="42" t="s">
-        <v>374</v>
+        <v>348</v>
       </c>
       <c r="K21" s="46" t="s">
-        <v>413</v>
+        <v>387</v>
       </c>
       <c r="M21" t="s">
         <v>197</v>
@@ -5320,10 +5782,10 @@
         <v>148</v>
       </c>
       <c r="D22" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E22" s="42" t="s">
-        <v>377</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" spans="2:14" ht="16.5" thickTop="1" thickBot="1">
@@ -5334,10 +5796,10 @@
         <v>148</v>
       </c>
       <c r="D23" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E23" s="42" t="s">
-        <v>377</v>
+        <v>351</v>
       </c>
     </row>
     <row r="24" spans="2:14" ht="16.5" thickTop="1" thickBot="1">
@@ -5348,10 +5810,10 @@
         <v>148</v>
       </c>
       <c r="D24" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E24" s="42" t="s">
-        <v>378</v>
+        <v>352</v>
       </c>
       <c r="M24" t="s">
         <v>269</v>
@@ -5365,10 +5827,10 @@
         <v>148</v>
       </c>
       <c r="D25" s="42" t="s">
-        <v>370</v>
+        <v>344</v>
       </c>
       <c r="E25" s="42" t="s">
-        <v>379</v>
+        <v>353</v>
       </c>
       <c r="M25" t="s">
         <v>270</v>
@@ -5551,142 +6013,998 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15485827-58BF-48F2-B6AA-CA9493DA6400}">
-  <dimension ref="A2:B37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8026CEE6-0CF4-4B9F-AD83-C320C38CE0F4}">
+  <dimension ref="A2:P54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="62.28515625" customWidth="1"/>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" customWidth="1"/>
+    <col min="6" max="6" width="30.140625" customWidth="1"/>
+    <col min="8" max="8" width="33.85546875" customWidth="1"/>
+    <col min="10" max="11" width="37" customWidth="1"/>
+    <col min="12" max="12" width="60.42578125" customWidth="1"/>
+    <col min="15" max="15" width="36.140625" customWidth="1"/>
+    <col min="16" max="16" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>284</v>
-      </c>
-      <c r="B18" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="A29" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1">
-      <c r="A33" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1">
-      <c r="A34" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1">
-      <c r="A35" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1">
-      <c r="A36" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1">
-      <c r="A37" t="s">
-        <v>296</v>
-      </c>
+    <row r="2" spans="1:16">
+      <c r="A2" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="H2" s="10"/>
+      <c r="J2" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="O2" s="9"/>
+    </row>
+    <row r="3" spans="1:16" ht="15.75" thickBot="1">
+      <c r="B3" s="49" t="s">
+        <v>389</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>450</v>
+      </c>
+      <c r="D3" s="49" t="s">
+        <v>390</v>
+      </c>
+      <c r="E3" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>391</v>
+      </c>
+      <c r="G3" s="49" t="s">
+        <v>392</v>
+      </c>
+      <c r="I3" s="50" t="s">
+        <v>452</v>
+      </c>
+      <c r="J3" s="50" t="s">
+        <v>491</v>
+      </c>
+      <c r="K3" s="50" t="s">
+        <v>492</v>
+      </c>
+      <c r="L3" s="50" t="s">
+        <v>528</v>
+      </c>
+      <c r="N3" s="50" t="s">
+        <v>452</v>
+      </c>
+      <c r="O3" s="50" t="s">
+        <v>491</v>
+      </c>
+      <c r="P3" s="50" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="15.75" thickTop="1">
+      <c r="B4" s="48" t="s">
+        <v>393</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>299</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="E4" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>440</v>
+      </c>
+      <c r="G4" s="48" t="s">
+        <v>444</v>
+      </c>
+      <c r="I4" s="69" t="s">
+        <v>453</v>
+      </c>
+      <c r="J4" s="69" t="s">
+        <v>454</v>
+      </c>
+      <c r="K4" s="52"/>
+      <c r="L4" s="52" t="s">
+        <v>526</v>
+      </c>
+      <c r="N4" s="71" t="s">
+        <v>471</v>
+      </c>
+      <c r="O4" s="69" t="s">
+        <v>469</v>
+      </c>
+      <c r="P4" s="70" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="B5" s="48" t="s">
+        <v>394</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>311</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="E5" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>441</v>
+      </c>
+      <c r="G5" s="48" t="s">
+        <v>444</v>
+      </c>
+      <c r="I5" s="70"/>
+      <c r="J5" s="71" t="s">
+        <v>455</v>
+      </c>
+      <c r="K5" s="52"/>
+      <c r="N5" s="70"/>
+      <c r="O5" s="71" t="s">
+        <v>472</v>
+      </c>
+      <c r="P5" s="70" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="P6" s="70" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="B7" s="48" t="s">
+        <v>395</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>406</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="E7" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="F7" s="48" t="s">
+        <v>442</v>
+      </c>
+      <c r="G7" s="48" t="s">
+        <v>445</v>
+      </c>
+      <c r="N7" s="70"/>
+      <c r="O7" s="70"/>
+      <c r="P7" s="70" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="B8" s="48" t="s">
+        <v>396</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>407</v>
+      </c>
+      <c r="D8" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="E8" s="48" t="s">
+        <v>405</v>
+      </c>
+      <c r="F8" s="48" t="s">
+        <v>443</v>
+      </c>
+      <c r="G8" s="48" t="s">
+        <v>444</v>
+      </c>
+      <c r="I8" s="66" t="s">
+        <v>457</v>
+      </c>
+      <c r="J8" s="66" t="s">
+        <v>454</v>
+      </c>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55" t="s">
+        <v>527</v>
+      </c>
+      <c r="N8" s="70"/>
+      <c r="O8" s="69" t="s">
+        <v>473</v>
+      </c>
+      <c r="P8" s="70" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="I9" s="68"/>
+      <c r="J9" s="67" t="s">
+        <v>458</v>
+      </c>
+      <c r="K9" s="55"/>
+      <c r="L9" s="55"/>
+      <c r="N9" s="70"/>
+      <c r="O9" s="71" t="s">
+        <v>474</v>
+      </c>
+      <c r="P9" s="70" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="B10" s="48" t="s">
+        <v>397</v>
+      </c>
+      <c r="C10" s="48" t="s">
+        <v>408</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>416</v>
+      </c>
+      <c r="E10" s="48" t="s">
+        <v>424</v>
+      </c>
+      <c r="F10" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="G10" s="48" t="s">
+        <v>446</v>
+      </c>
+      <c r="I10" s="68"/>
+      <c r="J10" s="68" t="s">
+        <v>456</v>
+      </c>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="N10" s="70"/>
+      <c r="O10" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="P10" s="70" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="B11" s="48" t="s">
+        <v>398</v>
+      </c>
+      <c r="C11" s="48" t="s">
+        <v>409</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>417</v>
+      </c>
+      <c r="E11" s="48" t="s">
+        <v>425</v>
+      </c>
+      <c r="F11" s="48" t="s">
+        <v>433</v>
+      </c>
+      <c r="G11" s="48" t="s">
+        <v>446</v>
+      </c>
+      <c r="N11" s="70"/>
+      <c r="O11" s="70"/>
+      <c r="P11" s="70"/>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="B12" s="48" t="s">
+        <v>399</v>
+      </c>
+      <c r="C12" s="48" t="s">
+        <v>410</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>418</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>426</v>
+      </c>
+      <c r="F12" s="48" t="s">
+        <v>434</v>
+      </c>
+      <c r="G12" s="48" t="s">
+        <v>446</v>
+      </c>
+      <c r="I12" s="63" t="s">
+        <v>459</v>
+      </c>
+      <c r="J12" s="63" t="s">
+        <v>454</v>
+      </c>
+      <c r="K12" s="64" t="s">
+        <v>493</v>
+      </c>
+      <c r="L12" s="64" t="s">
+        <v>517</v>
+      </c>
+      <c r="N12" s="70"/>
+      <c r="O12" s="69" t="s">
+        <v>475</v>
+      </c>
+      <c r="P12" s="70"/>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="48"/>
+      <c r="I13" s="65"/>
+      <c r="J13" s="64" t="s">
+        <v>460</v>
+      </c>
+      <c r="K13" s="64" t="s">
+        <v>494</v>
+      </c>
+      <c r="L13" s="64" t="s">
+        <v>518</v>
+      </c>
+      <c r="N13" s="70"/>
+      <c r="O13" s="71" t="s">
+        <v>476</v>
+      </c>
+      <c r="P13" s="70"/>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="B14" s="48" t="s">
+        <v>400</v>
+      </c>
+      <c r="C14" s="48" t="s">
+        <v>411</v>
+      </c>
+      <c r="D14" s="48" t="s">
+        <v>419</v>
+      </c>
+      <c r="E14" s="48" t="s">
+        <v>427</v>
+      </c>
+      <c r="F14" s="48" t="s">
+        <v>435</v>
+      </c>
+      <c r="G14" s="48" t="s">
+        <v>447</v>
+      </c>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65" t="s">
+        <v>456</v>
+      </c>
+      <c r="K14" s="64" t="s">
+        <v>497</v>
+      </c>
+      <c r="L14" s="64" t="s">
+        <v>494</v>
+      </c>
+      <c r="N14" s="70"/>
+      <c r="O14" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="P14" s="70"/>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="B15" s="48" t="s">
+        <v>401</v>
+      </c>
+      <c r="C15" s="48" t="s">
+        <v>412</v>
+      </c>
+      <c r="D15" s="48" t="s">
+        <v>420</v>
+      </c>
+      <c r="E15" s="48" t="s">
+        <v>428</v>
+      </c>
+      <c r="F15" s="48" t="s">
+        <v>436</v>
+      </c>
+      <c r="G15" s="48" t="s">
+        <v>448</v>
+      </c>
+      <c r="I15" s="65"/>
+      <c r="J15" s="65"/>
+      <c r="K15" s="64" t="s">
+        <v>495</v>
+      </c>
+      <c r="L15" s="64" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="B16" s="48" t="s">
+        <v>402</v>
+      </c>
+      <c r="C16" s="48" t="s">
+        <v>413</v>
+      </c>
+      <c r="D16" s="48" t="s">
+        <v>421</v>
+      </c>
+      <c r="E16" s="48" t="s">
+        <v>429</v>
+      </c>
+      <c r="F16" s="48" t="s">
+        <v>437</v>
+      </c>
+      <c r="G16" s="48" t="s">
+        <v>448</v>
+      </c>
+      <c r="I16" s="65"/>
+      <c r="J16" s="63" t="s">
+        <v>461</v>
+      </c>
+      <c r="K16" s="64" t="s">
+        <v>496</v>
+      </c>
+      <c r="L16" s="64" t="s">
+        <v>520</v>
+      </c>
+      <c r="N16" s="54" t="s">
+        <v>477</v>
+      </c>
+      <c r="O16" s="54" t="s">
+        <v>461</v>
+      </c>
+      <c r="P16" s="68" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16">
+      <c r="B17" s="48" t="s">
+        <v>403</v>
+      </c>
+      <c r="C17" s="48" t="s">
+        <v>414</v>
+      </c>
+      <c r="D17" s="48" t="s">
+        <v>422</v>
+      </c>
+      <c r="E17" s="48" t="s">
+        <v>430</v>
+      </c>
+      <c r="F17" s="48" t="s">
+        <v>438</v>
+      </c>
+      <c r="G17" s="48" t="s">
+        <v>447</v>
+      </c>
+      <c r="I17" s="65"/>
+      <c r="J17" s="64" t="s">
+        <v>462</v>
+      </c>
+      <c r="K17" s="65"/>
+      <c r="L17" s="65" t="s">
+        <v>521</v>
+      </c>
+      <c r="N17" s="56"/>
+      <c r="O17" s="55" t="s">
+        <v>478</v>
+      </c>
+      <c r="P17" s="68" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16">
+      <c r="B18" s="48" t="s">
+        <v>404</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>415</v>
+      </c>
+      <c r="D18" s="48" t="s">
+        <v>423</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>431</v>
+      </c>
+      <c r="F18" s="48" t="s">
+        <v>439</v>
+      </c>
+      <c r="G18" s="48" t="s">
+        <v>449</v>
+      </c>
+      <c r="I18" s="65"/>
+      <c r="J18" s="65" t="s">
+        <v>456</v>
+      </c>
+      <c r="K18" s="65"/>
+      <c r="L18" s="65" t="s">
+        <v>496</v>
+      </c>
+      <c r="N18" s="56"/>
+      <c r="O18" s="56" t="s">
+        <v>456</v>
+      </c>
+      <c r="P18" s="68" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16">
+      <c r="N19" s="56"/>
+      <c r="O19" s="56"/>
+      <c r="P19" s="68" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16">
+      <c r="I20" s="60" t="s">
+        <v>463</v>
+      </c>
+      <c r="J20" s="60" t="s">
+        <v>454</v>
+      </c>
+      <c r="K20" s="61" t="s">
+        <v>493</v>
+      </c>
+      <c r="L20" s="62" t="s">
+        <v>517</v>
+      </c>
+      <c r="N20" s="56"/>
+      <c r="O20" s="54" t="s">
+        <v>469</v>
+      </c>
+      <c r="P20" s="68" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16">
+      <c r="I21" s="62"/>
+      <c r="J21" s="61" t="s">
+        <v>464</v>
+      </c>
+      <c r="K21" s="61" t="s">
+        <v>494</v>
+      </c>
+      <c r="L21" s="62" t="s">
+        <v>524</v>
+      </c>
+      <c r="N21" s="56"/>
+      <c r="O21" s="55" t="s">
+        <v>479</v>
+      </c>
+      <c r="P21" s="68" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16">
+      <c r="I22" s="62"/>
+      <c r="J22" s="62" t="s">
+        <v>456</v>
+      </c>
+      <c r="K22" s="61" t="s">
+        <v>498</v>
+      </c>
+      <c r="L22" s="62" t="s">
+        <v>494</v>
+      </c>
+      <c r="N22" s="56"/>
+      <c r="O22" s="56" t="s">
+        <v>456</v>
+      </c>
+      <c r="P22" s="56"/>
+    </row>
+    <row r="23" spans="2:16">
+      <c r="I23" s="62"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="61" t="s">
+        <v>499</v>
+      </c>
+      <c r="L23" s="62" t="s">
+        <v>519</v>
+      </c>
+      <c r="N23" s="56"/>
+      <c r="O23" s="56"/>
+      <c r="P23" s="56"/>
+    </row>
+    <row r="24" spans="2:16">
+      <c r="I24" s="62"/>
+      <c r="J24" s="60" t="s">
+        <v>461</v>
+      </c>
+      <c r="K24" s="61" t="s">
+        <v>496</v>
+      </c>
+      <c r="L24" s="62" t="s">
+        <v>520</v>
+      </c>
+      <c r="N24" s="56"/>
+      <c r="O24" s="54" t="s">
+        <v>475</v>
+      </c>
+      <c r="P24" s="56"/>
+    </row>
+    <row r="25" spans="2:16">
+      <c r="I25" s="62"/>
+      <c r="J25" s="61" t="s">
+        <v>465</v>
+      </c>
+      <c r="K25" s="62"/>
+      <c r="L25" s="62" t="s">
+        <v>525</v>
+      </c>
+      <c r="N25" s="56"/>
+      <c r="O25" s="55" t="s">
+        <v>480</v>
+      </c>
+      <c r="P25" s="56"/>
+    </row>
+    <row r="26" spans="2:16">
+      <c r="I26" s="62"/>
+      <c r="J26" s="62" t="s">
+        <v>456</v>
+      </c>
+      <c r="K26" s="62"/>
+      <c r="L26" s="62" t="s">
+        <v>496</v>
+      </c>
+      <c r="N26" s="56"/>
+      <c r="O26" s="56" t="s">
+        <v>456</v>
+      </c>
+      <c r="P26" s="56"/>
+    </row>
+    <row r="28" spans="2:16">
+      <c r="I28" s="57" t="s">
+        <v>466</v>
+      </c>
+      <c r="J28" s="57" t="s">
+        <v>454</v>
+      </c>
+      <c r="K28" s="58" t="s">
+        <v>493</v>
+      </c>
+      <c r="L28" s="58" t="s">
+        <v>517</v>
+      </c>
+      <c r="N28" s="63" t="s">
+        <v>481</v>
+      </c>
+      <c r="O28" s="63" t="s">
+        <v>461</v>
+      </c>
+      <c r="P28" s="65" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16">
+      <c r="I29" s="59"/>
+      <c r="J29" s="58" t="s">
+        <v>467</v>
+      </c>
+      <c r="K29" s="58" t="s">
+        <v>494</v>
+      </c>
+      <c r="L29" s="58" t="s">
+        <v>522</v>
+      </c>
+      <c r="N29" s="65"/>
+      <c r="O29" s="64" t="s">
+        <v>482</v>
+      </c>
+      <c r="P29" s="65" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16">
+      <c r="I30" s="59"/>
+      <c r="J30" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="K30" s="58" t="s">
+        <v>500</v>
+      </c>
+      <c r="L30" s="58" t="s">
+        <v>494</v>
+      </c>
+      <c r="N30" s="65"/>
+      <c r="O30" s="65" t="s">
+        <v>456</v>
+      </c>
+      <c r="P30" s="65" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16">
+      <c r="I31" s="59"/>
+      <c r="J31" s="59"/>
+      <c r="K31" s="58" t="s">
+        <v>501</v>
+      </c>
+      <c r="L31" s="58" t="s">
+        <v>519</v>
+      </c>
+      <c r="N31" s="65"/>
+      <c r="O31" s="65"/>
+      <c r="P31" s="65" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16">
+      <c r="I32" s="59"/>
+      <c r="J32" s="57" t="s">
+        <v>461</v>
+      </c>
+      <c r="K32" s="58" t="s">
+        <v>496</v>
+      </c>
+      <c r="L32" s="58" t="s">
+        <v>520</v>
+      </c>
+      <c r="N32" s="65"/>
+      <c r="O32" s="63" t="s">
+        <v>483</v>
+      </c>
+      <c r="P32" s="65" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="33" spans="9:16">
+      <c r="I33" s="59"/>
+      <c r="J33" s="58" t="s">
+        <v>468</v>
+      </c>
+      <c r="K33" s="59"/>
+      <c r="L33" s="58" t="s">
+        <v>523</v>
+      </c>
+      <c r="N33" s="65"/>
+      <c r="O33" s="64" t="s">
+        <v>484</v>
+      </c>
+      <c r="P33" s="65" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="34" spans="9:16">
+      <c r="I34" s="59"/>
+      <c r="J34" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="K34" s="58"/>
+      <c r="L34" s="58" t="s">
+        <v>496</v>
+      </c>
+      <c r="N34" s="65"/>
+      <c r="O34" s="65" t="s">
+        <v>456</v>
+      </c>
+      <c r="P34" s="65"/>
+    </row>
+    <row r="35" spans="9:16">
+      <c r="I35" s="59"/>
+      <c r="J35" s="59"/>
+      <c r="K35" s="58"/>
+      <c r="L35" s="58"/>
+      <c r="N35" s="65"/>
+      <c r="O35" s="65"/>
+      <c r="P35" s="65"/>
+    </row>
+    <row r="36" spans="9:16">
+      <c r="I36" s="59"/>
+      <c r="J36" s="57" t="s">
+        <v>469</v>
+      </c>
+      <c r="K36" s="59"/>
+      <c r="L36" s="59"/>
+      <c r="N36" s="65"/>
+      <c r="O36" s="63" t="s">
+        <v>475</v>
+      </c>
+      <c r="P36" s="65"/>
+    </row>
+    <row r="37" spans="9:16">
+      <c r="I37" s="59"/>
+      <c r="J37" s="58" t="s">
+        <v>470</v>
+      </c>
+      <c r="K37" s="59"/>
+      <c r="L37" s="59"/>
+      <c r="N37" s="65"/>
+      <c r="O37" s="64" t="s">
+        <v>485</v>
+      </c>
+      <c r="P37" s="65"/>
+    </row>
+    <row r="38" spans="9:16">
+      <c r="I38" s="59"/>
+      <c r="J38" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="K38" s="58"/>
+      <c r="L38" s="58"/>
+      <c r="N38" s="65"/>
+      <c r="O38" s="65" t="s">
+        <v>456</v>
+      </c>
+      <c r="P38" s="65"/>
+    </row>
+    <row r="39" spans="9:16">
+      <c r="K39" s="51"/>
+      <c r="L39" s="51"/>
+    </row>
+    <row r="40" spans="9:16">
+      <c r="I40" s="69" t="s">
+        <v>99</v>
+      </c>
+      <c r="J40" s="69" t="s">
+        <v>469</v>
+      </c>
+      <c r="K40" s="52"/>
+      <c r="L40" s="52"/>
+      <c r="N40" s="57" t="s">
+        <v>486</v>
+      </c>
+      <c r="O40" s="57" t="s">
+        <v>461</v>
+      </c>
+      <c r="P40" s="59" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="41" spans="9:16">
+      <c r="I41" s="70"/>
+      <c r="J41" s="71" t="s">
+        <v>530</v>
+      </c>
+      <c r="K41" s="52"/>
+      <c r="L41" s="52"/>
+      <c r="N41" s="59"/>
+      <c r="O41" s="58" t="s">
+        <v>487</v>
+      </c>
+      <c r="P41" s="59" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="42" spans="9:16">
+      <c r="I42" s="70"/>
+      <c r="J42" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="K42" s="53"/>
+      <c r="L42" s="53"/>
+      <c r="N42" s="59"/>
+      <c r="O42" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="P42" s="59" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="43" spans="9:16">
+      <c r="N43" s="59"/>
+      <c r="O43" s="59"/>
+      <c r="P43" s="59" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="44" spans="9:16">
+      <c r="I44" s="66" t="s">
+        <v>101</v>
+      </c>
+      <c r="J44" s="66" t="s">
+        <v>469</v>
+      </c>
+      <c r="K44" s="55"/>
+      <c r="L44" s="55" t="s">
+        <v>529</v>
+      </c>
+      <c r="N44" s="59"/>
+      <c r="O44" s="57" t="s">
+        <v>469</v>
+      </c>
+      <c r="P44" s="59" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="45" spans="9:16">
+      <c r="I45" s="68"/>
+      <c r="J45" s="67" t="s">
+        <v>531</v>
+      </c>
+      <c r="K45" s="55"/>
+      <c r="L45" s="55"/>
+      <c r="N45" s="59"/>
+      <c r="O45" s="58" t="s">
+        <v>488</v>
+      </c>
+      <c r="P45" s="59" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="46" spans="9:16">
+      <c r="I46" s="68"/>
+      <c r="J46" s="68" t="s">
+        <v>456</v>
+      </c>
+      <c r="K46" s="56"/>
+      <c r="L46" s="56"/>
+      <c r="N46" s="59"/>
+      <c r="O46" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="P46" s="59"/>
+    </row>
+    <row r="47" spans="9:16">
+      <c r="N47" s="59"/>
+      <c r="O47" s="59"/>
+      <c r="P47" s="59"/>
+    </row>
+    <row r="48" spans="9:16">
+      <c r="N48" s="59"/>
+      <c r="O48" s="57" t="s">
+        <v>473</v>
+      </c>
+      <c r="P48" s="59"/>
+    </row>
+    <row r="49" spans="14:16">
+      <c r="N49" s="59"/>
+      <c r="O49" s="58" t="s">
+        <v>489</v>
+      </c>
+      <c r="P49" s="59"/>
+    </row>
+    <row r="50" spans="14:16">
+      <c r="N50" s="59"/>
+      <c r="O50" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="P50" s="59"/>
+    </row>
+    <row r="51" spans="14:16">
+      <c r="N51" s="59"/>
+      <c r="O51" s="59"/>
+      <c r="P51" s="59"/>
+    </row>
+    <row r="52" spans="14:16">
+      <c r="N52" s="59"/>
+      <c r="O52" s="57" t="s">
+        <v>475</v>
+      </c>
+      <c r="P52" s="59"/>
+    </row>
+    <row r="53" spans="14:16">
+      <c r="N53" s="59"/>
+      <c r="O53" s="58" t="s">
+        <v>490</v>
+      </c>
+      <c r="P53" s="59"/>
+    </row>
+    <row r="54" spans="14:16">
+      <c r="N54" s="59"/>
+      <c r="O54" s="59" t="s">
+        <v>456</v>
+      </c>
+      <c r="P54" s="59"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Réalisation de la 3eme partie du projet
</commit_message>
<xml_diff>
--- a/docs/Resume_Table_addressage.xlsx
+++ b/docs/Resume_Table_addressage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\njlid\Desktop\cnam\cnam-24-25\RSX103\portfolio\Secure-Entrepise-Network-Architecture\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFD6085-A3BC-4AD9-812E-027D0A082A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49A34BB-4A9F-4E8D-AF11-9B913DC60CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="15105" windowHeight="15585" firstSheet="2" activeTab="6" xr2:uid="{95F63387-710A-4DE0-80EC-A390F828E8CA}"/>
+    <workbookView xWindow="-705" yWindow="45" windowWidth="18225" windowHeight="14895" firstSheet="4" activeTab="5" xr2:uid="{95F63387-710A-4DE0-80EC-A390F828E8CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil3" sheetId="3" r:id="rId1"/>
@@ -19,9 +19,12 @@
     <sheet name="DHCP" sheetId="5" r:id="rId4"/>
     <sheet name="NAT" sheetId="6" r:id="rId5"/>
     <sheet name="ACL" sheetId="4" r:id="rId6"/>
-    <sheet name="Plan d'adressage R Op" sheetId="8" r:id="rId7"/>
+    <sheet name="Routage IP (ospf+static)" sheetId="8" r:id="rId7"/>
+    <sheet name="MPLS" sheetId="9" r:id="rId8"/>
+    <sheet name="Feuil2" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="575">
   <si>
     <t>Site</t>
   </si>
@@ -1890,33 +1893,12 @@
     <t>access-list 100 deny ip 192.168.2.32 0.0.0.31 192.168.2.0 0.0.0.31</t>
   </si>
   <si>
-    <t>access-list 101 deny ip 192.168.1.64 0.0.0.7 123.1.1.162 0.0.0.15</t>
-  </si>
-  <si>
-    <t>access-list 101 deny ip 192.168.2.64 0.0.0.7 123.2.2.162 0.0.0.7</t>
-  </si>
-  <si>
-    <t>access-list 101 deny ip 123.1.1.162 0.0.0.15 192.168.1.64 0.0.0.7</t>
-  </si>
-  <si>
-    <t>access-list 101 deny ip 123.2.2.162 0.0.0.7 192.168.2.64 0.0.0.7</t>
-  </si>
-  <si>
     <t>Configuration des ACL sur les routeurs de chacun des sites</t>
   </si>
   <si>
     <t>Application des ACL sur les interfaces des routeurs R1 et R2</t>
   </si>
   <si>
-    <t xml:space="preserve">interface e1/1.10 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">interface e1/1.20 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">interface e1/1.31 </t>
-  </si>
-  <si>
     <t>ip access-group 101 in</t>
   </si>
   <si>
@@ -2362,13 +2344,213 @@
   </si>
   <si>
     <t>#  network 12.0.0.12 0.0.0.3 area 0</t>
+  </si>
+  <si>
+    <t>Configuration MPLS (cef, ldp et activation sur interfaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration </t>
+  </si>
+  <si>
+    <t>R1/R2/RF2</t>
+  </si>
+  <si>
+    <t>ip cef</t>
+  </si>
+  <si>
+    <t>mpls ip</t>
+  </si>
+  <si>
+    <t>mpls label protocol ldp</t>
+  </si>
+  <si>
+    <t>interface e1/0</t>
+  </si>
+  <si>
+    <t>interface e1/2</t>
+  </si>
+  <si>
+    <t>interface e1/3</t>
+  </si>
+  <si>
+    <t>RO3</t>
+  </si>
+  <si>
+    <t>Sur R1</t>
+  </si>
+  <si>
+    <t>configuration terminal</t>
+  </si>
+  <si>
+    <t>interface e1/2.10</t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sur R2 </t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.1</t>
+  </si>
+  <si>
+    <t>interface e1/2.20</t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.2</t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.3</t>
+  </si>
+  <si>
+    <t>interface e1/2.31</t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.4</t>
+  </si>
+  <si>
+    <t>ip address 192.168.0.5</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Etape 1 :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> définir les sous interfaces vertuelles</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Réseau : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="5"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>192.168.0.0/24</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Etape 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : définir des routes statiques</t>
+    </r>
+  </si>
+  <si>
+    <t>Cible</t>
+  </si>
+  <si>
+    <t>Commande</t>
+  </si>
+  <si>
+    <t>ip route 192.168.2.0 255.255.255.224 192.168.0.1</t>
+  </si>
+  <si>
+    <t>ip route 192.168.2.32 255.255.255.224 192.168.0.3</t>
+  </si>
+  <si>
+    <t>ip route 192.168.2.64 255.255.255.248 192.168.0.5</t>
+  </si>
+  <si>
+    <t>ip route 192.168.1.0 255.255.255.224 192.168.0.0</t>
+  </si>
+  <si>
+    <t>ip route 192.168.1.32 255.255.255.224 192.168.0.2</t>
+  </si>
+  <si>
+    <t>ip route 192.168.1.64 255.255.255.248 192.168.0.4</t>
+  </si>
+  <si>
+    <t>(en mode configuration)</t>
+  </si>
+  <si>
+    <t>access-list 100 deny ip 192.168.1.0 0.0.0.31 192.168.2.32 0.0.0.31</t>
+  </si>
+  <si>
+    <t>access-list 100 deny ip 192.168.1.32 0.0.0.31 192.168.2.0 0.0.0.31</t>
+  </si>
+  <si>
+    <t>access-list 100 deny ip 192.168.2.0 0.0.0.31 192.168.1.32 0.0.0.31</t>
+  </si>
+  <si>
+    <t>access-list 100 deny ip 192.168.2.32 0.0.0.31 192.168.1.0 0.0.0.31</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 192.168.1.64 0.0.0.7 123.1.1.160 0.0.0.15</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 192.168.1.64 0.0.0.7 123.2.2.160 0.0.0.7</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 123.1.1.160 0.0.0.15 192.168.1.64 0.0.0.7</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 123.1.1.160 0.0.0.15 192.168.2.64 0.0.0.7</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 192.168.2.64 0.0.0.7 123.2.2.160 0.0.0.7</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 192.168.2.64 0.0.0.7 123.1.1.160 0.0.0.15</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 123.2.2.160 0.0.0.7 192.168.1.64 0.0.0.7</t>
+  </si>
+  <si>
+    <t>access-list 101 deny ip 123.2.2.160 0.0.0.7 192.168.2.64 0.0.0.7</t>
+  </si>
+  <si>
+    <t>interface e1/1.10    (e1/2.10)</t>
+  </si>
+  <si>
+    <t>interface e1/1.20    (e1/2.20)</t>
+  </si>
+  <si>
+    <t>interface e1/1.31  (e1/2.31)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2560,8 +2742,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2665,8 +2863,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -2770,8 +2974,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="12">
+  <cellStyleXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
@@ -2784,8 +2999,10 @@
     <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="25" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2892,10 +3109,17 @@
     <xf numFmtId="0" fontId="17" fillId="14" borderId="8" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="14" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="12"/>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="11"/>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="13"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="13" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" xfId="11" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" xfId="8" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="12">
+  <cellStyles count="14">
     <cellStyle name="20 % - Accent1" xfId="11" builtinId="30"/>
     <cellStyle name="20 % - Accent2" xfId="8" builtinId="34"/>
+    <cellStyle name="20 % - Accent3" xfId="13" builtinId="38"/>
     <cellStyle name="20 % - Accent6" xfId="9" builtinId="50"/>
     <cellStyle name="40 % - Accent1" xfId="6" builtinId="31"/>
     <cellStyle name="Accent1" xfId="5" builtinId="29"/>
@@ -2906,8 +3130,46 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Satisfaisant" xfId="1" builtinId="26"/>
     <cellStyle name="Sortie" xfId="10" builtinId="21"/>
+    <cellStyle name="Total" xfId="12" builtinId="25"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2995,6 +3257,38 @@
 </table>
 </file>
 
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{D9AC8841-54A0-4782-A51E-695310E5C387}" name="Tableau13" displayName="Tableau13" ref="C1:C14" totalsRowShown="0" headerRowDxfId="1" headerRowCellStyle="20 % - Accent1">
+  <autoFilter ref="C1:C14" xr:uid="{D9AC8841-54A0-4782-A51E-695310E5C387}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{DABB31BE-C690-4521-BFFB-6CB68E58B3C3}" name="Sur R1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{D15827C6-710B-417A-AB41-63957F35ABFC}" name="Tableau14" displayName="Tableau14" ref="E1:E14" totalsRowShown="0" headerRowDxfId="0" headerRowCellStyle="20 % - Accent2">
+  <autoFilter ref="E1:E14" xr:uid="{D15827C6-710B-417A-AB41-63957F35ABFC}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{4DD007D3-AC64-4650-8A07-7D03FD29AFA7}" name="Sur R2 "/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{F66C624F-7D54-4ABE-A3C7-00AD35D89FCC}" name="Tableau16" displayName="Tableau16" ref="H1:J8" totalsRowShown="0">
+  <autoFilter ref="H1:J8" xr:uid="{F66C624F-7D54-4ABE-A3C7-00AD35D89FCC}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{7E0E953D-3764-4BA3-A446-4FC63F979D8D}" name="Routeur"/>
+    <tableColumn id="2" xr3:uid="{9BD4B5A2-B8FB-4225-94C8-EC65EDF51C2F}" name="Cible"/>
+    <tableColumn id="3" xr3:uid="{86A48E47-5F59-431D-8EE2-29150C69D7EE}" name="Commande"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{D709B4FA-1F58-450F-A0F3-0A782D67D3CE}" name="Tableau6" displayName="Tableau6" ref="D25:G41" totalsRowShown="0">
   <autoFilter ref="D25:G41" xr:uid="{D709B4FA-1F58-450F-A0F3-0A782D67D3CE}"/>
@@ -3014,7 +3308,7 @@
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D1948EA8-C458-48F1-8035-5E952203BB10}" name="Nom VLAN"/>
     <tableColumn id="2" xr3:uid="{D0B8288D-B83B-4F67-BCB2-F0EC4644D3A0}" name="Département"/>
-    <tableColumn id="3" xr3:uid="{7C52E67F-410F-4DDB-86CC-9EA5B244BDA6}" name="ID" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{7C52E67F-410F-4DDB-86CC-9EA5B244BDA6}" name="ID" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{B52AF3C8-6212-4937-B144-96E08370F0F8}" name="Plage IP -site1"/>
     <tableColumn id="5" xr3:uid="{168FD971-2400-4505-AEE0-4E5D64BA9862}" name="Switch"/>
     <tableColumn id="6" xr3:uid="{23C78678-D8AF-4DB2-9C47-01BD3ED87E6D}" name="Interface"/>
@@ -5393,13 +5687,16 @@
         <v>358</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="T4" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="5" spans="2:20">
+      <c r="H5" t="s">
+        <v>559</v>
+      </c>
       <c r="M5" t="s">
         <v>222</v>
       </c>
@@ -5430,7 +5727,7 @@
         <v>361</v>
       </c>
       <c r="K6" s="47" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="M6" t="s">
         <v>149</v>
@@ -5478,14 +5775,14 @@
       </c>
       <c r="G8" s="45"/>
       <c r="H8" s="45" t="s">
-        <v>373</v>
+        <v>560</v>
       </c>
       <c r="I8" s="45" t="s">
-        <v>374</v>
+        <v>562</v>
       </c>
       <c r="J8" s="45"/>
       <c r="K8" s="46" t="s">
-        <v>381</v>
+        <v>572</v>
       </c>
       <c r="M8" t="s">
         <v>157</v>
@@ -5498,13 +5795,10 @@
       <c r="E9" s="42"/>
       <c r="G9" s="45"/>
       <c r="H9" s="45" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="I9" s="45" t="s">
-        <v>364</v>
-      </c>
-      <c r="J9" s="45" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="K9" s="46" t="s">
         <v>234</v>
@@ -5527,8 +5821,12 @@
         <v>354</v>
       </c>
       <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
+      <c r="H10" s="45" t="s">
+        <v>561</v>
+      </c>
+      <c r="I10" s="45" t="s">
+        <v>563</v>
+      </c>
       <c r="J10" s="45"/>
       <c r="K10" s="46"/>
     </row>
@@ -5545,20 +5843,18 @@
       <c r="E11" s="42" t="s">
         <v>356</v>
       </c>
-      <c r="G11" s="44">
-        <v>101</v>
-      </c>
+      <c r="G11" s="45"/>
       <c r="H11" s="45" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="I11" s="45" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="J11" s="45" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="K11" s="46" t="s">
-        <v>382</v>
+        <v>573</v>
       </c>
       <c r="M11" t="s">
         <v>223</v>
@@ -5578,12 +5874,8 @@
         <v>355</v>
       </c>
       <c r="G12" s="45"/>
-      <c r="H12" s="45" t="s">
-        <v>377</v>
-      </c>
-      <c r="I12" s="45" t="s">
-        <v>378</v>
-      </c>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
       <c r="J12" s="45"/>
       <c r="K12" s="46" t="s">
         <v>234</v>
@@ -5605,14 +5897,18 @@
       <c r="E13" s="42" t="s">
         <v>357</v>
       </c>
-      <c r="G13" s="45"/>
+      <c r="G13" s="44">
+        <v>101</v>
+      </c>
       <c r="H13" s="45" t="s">
-        <v>366</v>
+        <v>564</v>
       </c>
       <c r="I13" s="45" t="s">
-        <v>366</v>
-      </c>
-      <c r="J13" s="45"/>
+        <v>568</v>
+      </c>
+      <c r="J13" s="45" t="s">
+        <v>367</v>
+      </c>
       <c r="K13" s="46"/>
       <c r="M13" t="s">
         <v>159</v>
@@ -5624,11 +5920,15 @@
       <c r="D14" s="42"/>
       <c r="E14" s="42"/>
       <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
+      <c r="H14" s="45" t="s">
+        <v>565</v>
+      </c>
+      <c r="I14" s="45" t="s">
+        <v>569</v>
+      </c>
       <c r="J14" s="45"/>
       <c r="K14" s="46" t="s">
-        <v>383</v>
+        <v>574</v>
       </c>
     </row>
     <row r="15" spans="2:20" ht="16.5" thickTop="1" thickBot="1">
@@ -5644,20 +5944,15 @@
       <c r="E15" s="42" t="s">
         <v>347</v>
       </c>
-      <c r="G15" s="44">
-        <v>102</v>
-      </c>
       <c r="H15" s="45" t="s">
-        <v>368</v>
+        <v>566</v>
       </c>
       <c r="I15" s="45" t="s">
-        <v>370</v>
-      </c>
-      <c r="J15" s="45" t="s">
-        <v>371</v>
-      </c>
+        <v>571</v>
+      </c>
+      <c r="J15" s="45"/>
       <c r="K15" s="46" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
     </row>
     <row r="16" spans="2:20" ht="16.5" thickTop="1" thickBot="1">
@@ -5675,10 +5970,10 @@
       </c>
       <c r="G16" s="45"/>
       <c r="H16" s="45" t="s">
-        <v>369</v>
+        <v>567</v>
       </c>
       <c r="I16" s="45" t="s">
-        <v>369</v>
+        <v>570</v>
       </c>
       <c r="J16" s="45"/>
       <c r="K16" s="46"/>
@@ -5692,11 +5987,15 @@
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
       <c r="G17" s="45"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="45"/>
+      <c r="H17" s="45" t="s">
+        <v>366</v>
+      </c>
+      <c r="I17" s="45" t="s">
+        <v>366</v>
+      </c>
       <c r="J17" s="45"/>
       <c r="K17" s="46" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="M17" t="s">
         <v>161</v>
@@ -5715,8 +6014,12 @@
       <c r="E18" s="42" t="s">
         <v>349</v>
       </c>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
       <c r="K18" s="46" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="M18" t="s">
         <v>162</v>
@@ -5735,6 +6038,18 @@
       <c r="E19" s="42" t="s">
         <v>350</v>
       </c>
+      <c r="G19" s="44">
+        <v>102</v>
+      </c>
+      <c r="H19" s="45" t="s">
+        <v>368</v>
+      </c>
+      <c r="I19" s="45" t="s">
+        <v>370</v>
+      </c>
+      <c r="J19" s="45" t="s">
+        <v>371</v>
+      </c>
       <c r="M19" t="s">
         <v>163</v>
       </c>
@@ -5750,8 +6065,16 @@
         <v>343</v>
       </c>
       <c r="E20" s="42"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45" t="s">
+        <v>369</v>
+      </c>
+      <c r="I20" s="45" t="s">
+        <v>369</v>
+      </c>
+      <c r="J20" s="45"/>
       <c r="K20" s="46" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
     </row>
     <row r="21" spans="2:14" ht="16.5" thickTop="1" thickBot="1">
@@ -5767,8 +6090,12 @@
       <c r="E21" s="42" t="s">
         <v>348</v>
       </c>
+      <c r="G21" s="45"/>
+      <c r="H21" s="45"/>
+      <c r="I21" s="45"/>
+      <c r="J21" s="45"/>
       <c r="K21" s="46" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
       <c r="M21" t="s">
         <v>197</v>
@@ -6031,11 +6358,11 @@
   <sheetData>
     <row r="2" spans="1:16">
       <c r="A2" s="10" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="H2" s="10"/>
       <c r="J2" s="9" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
@@ -6043,114 +6370,114 @@
     </row>
     <row r="3" spans="1:16" ht="15.75" thickBot="1">
       <c r="B3" s="49" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="E3" s="49" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="G3" s="49" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="I3" s="50" t="s">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="J3" s="50" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="K3" s="50" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="L3" s="50" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="N3" s="50" t="s">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="O3" s="50" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="P3" s="50" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" thickTop="1">
       <c r="B4" s="48" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="C4" s="48" t="s">
         <v>299</v>
       </c>
       <c r="D4" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E4" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="F4" s="48" t="s">
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="G4" s="48" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="I4" s="69" t="s">
-        <v>453</v>
+        <v>446</v>
       </c>
       <c r="J4" s="69" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="K4" s="52"/>
       <c r="L4" s="52" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="N4" s="71" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="O4" s="69" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="P4" s="70" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="B5" s="48" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="C5" s="48" t="s">
         <v>311</v>
       </c>
       <c r="D5" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E5" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="F5" s="48" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="G5" s="48" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="I5" s="70"/>
       <c r="J5" s="71" t="s">
-        <v>455</v>
+        <v>448</v>
       </c>
       <c r="K5" s="52"/>
       <c r="N5" s="70"/>
       <c r="O5" s="71" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="P5" s="70" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -6162,78 +6489,78 @@
       <c r="G6" s="48"/>
       <c r="I6" s="70"/>
       <c r="J6" s="70" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K6" s="53"/>
       <c r="L6" s="53"/>
       <c r="N6" s="70"/>
       <c r="O6" s="70" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P6" s="70" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7" spans="1:16">
       <c r="B7" s="48" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="C7" s="48" t="s">
-        <v>406</v>
+        <v>399</v>
       </c>
       <c r="D7" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E7" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="F7" s="48" t="s">
-        <v>442</v>
+        <v>435</v>
       </c>
       <c r="G7" s="48" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
       <c r="N7" s="70"/>
       <c r="O7" s="70"/>
       <c r="P7" s="70" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
     </row>
     <row r="8" spans="1:16">
       <c r="B8" s="48" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="C8" s="48" t="s">
-        <v>407</v>
+        <v>400</v>
       </c>
       <c r="D8" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="E8" s="48" t="s">
-        <v>405</v>
+        <v>398</v>
       </c>
       <c r="F8" s="48" t="s">
-        <v>443</v>
+        <v>436</v>
       </c>
       <c r="G8" s="48" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
       <c r="I8" s="66" t="s">
-        <v>457</v>
+        <v>450</v>
       </c>
       <c r="J8" s="66" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="K8" s="55"/>
       <c r="L8" s="55" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="N8" s="70"/>
       <c r="O8" s="69" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="P8" s="70" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -6245,69 +6572,69 @@
       <c r="G9" s="48"/>
       <c r="I9" s="68"/>
       <c r="J9" s="67" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K9" s="55"/>
       <c r="L9" s="55"/>
       <c r="N9" s="70"/>
       <c r="O9" s="71" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
       <c r="P9" s="70" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="10" spans="1:16">
       <c r="B10" s="48" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="C10" s="48" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="D10" s="48" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="F10" s="48" t="s">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="I10" s="68"/>
       <c r="J10" s="68" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K10" s="56"/>
       <c r="L10" s="56"/>
       <c r="N10" s="70"/>
       <c r="O10" s="70" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P10" s="70" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="B11" s="48" t="s">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="C11" s="48" t="s">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="D11" s="48" t="s">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="E11" s="48" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="F11" s="48" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="G11" s="48" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="N11" s="70"/>
       <c r="O11" s="70"/>
@@ -6315,38 +6642,38 @@
     </row>
     <row r="12" spans="1:16">
       <c r="B12" s="48" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="C12" s="48" t="s">
-        <v>410</v>
+        <v>403</v>
       </c>
       <c r="D12" s="48" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="E12" s="48" t="s">
-        <v>426</v>
+        <v>419</v>
       </c>
       <c r="F12" s="48" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
       <c r="G12" s="48" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="I12" s="63" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="J12" s="63" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="K12" s="64" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="L12" s="64" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="N12" s="70"/>
       <c r="O12" s="69" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="P12" s="70"/>
     </row>
@@ -6359,253 +6686,253 @@
       <c r="G13" s="48"/>
       <c r="I13" s="65"/>
       <c r="J13" s="64" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
       <c r="K13" s="64" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="L13" s="64" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N13" s="70"/>
       <c r="O13" s="71" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="P13" s="70"/>
     </row>
     <row r="14" spans="1:16">
       <c r="B14" s="48" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="D14" s="48" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="E14" s="48" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="F14" s="48" t="s">
-        <v>435</v>
+        <v>428</v>
       </c>
       <c r="G14" s="48" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="I14" s="65"/>
       <c r="J14" s="65" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K14" s="64" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="L14" s="64" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="N14" s="70"/>
       <c r="O14" s="70" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P14" s="70"/>
     </row>
     <row r="15" spans="1:16">
       <c r="B15" s="48" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="C15" s="48" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="D15" s="48" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="E15" s="48" t="s">
-        <v>428</v>
+        <v>421</v>
       </c>
       <c r="F15" s="48" t="s">
-        <v>436</v>
+        <v>429</v>
       </c>
       <c r="G15" s="48" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="I15" s="65"/>
       <c r="J15" s="65"/>
       <c r="K15" s="64" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L15" s="64" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
     </row>
     <row r="16" spans="1:16">
       <c r="B16" s="48" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="C16" s="48" t="s">
-        <v>413</v>
+        <v>406</v>
       </c>
       <c r="D16" s="48" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="E16" s="48" t="s">
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="F16" s="48" t="s">
-        <v>437</v>
+        <v>430</v>
       </c>
       <c r="G16" s="48" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="I16" s="65"/>
       <c r="J16" s="63" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="K16" s="64" t="s">
+        <v>489</v>
+      </c>
+      <c r="L16" s="64" t="s">
+        <v>513</v>
+      </c>
+      <c r="N16" s="54" t="s">
+        <v>470</v>
+      </c>
+      <c r="O16" s="54" t="s">
+        <v>454</v>
+      </c>
+      <c r="P16" s="68" t="s">
         <v>496</v>
-      </c>
-      <c r="L16" s="64" t="s">
-        <v>520</v>
-      </c>
-      <c r="N16" s="54" t="s">
-        <v>477</v>
-      </c>
-      <c r="O16" s="54" t="s">
-        <v>461</v>
-      </c>
-      <c r="P16" s="68" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="17" spans="2:16">
       <c r="B17" s="48" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>414</v>
+        <v>407</v>
       </c>
       <c r="D17" s="48" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="E17" s="48" t="s">
-        <v>430</v>
+        <v>423</v>
       </c>
       <c r="F17" s="48" t="s">
-        <v>438</v>
+        <v>431</v>
       </c>
       <c r="G17" s="48" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="I17" s="65"/>
       <c r="J17" s="64" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
       <c r="K17" s="65"/>
       <c r="L17" s="65" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="N17" s="56"/>
       <c r="O17" s="55" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="P17" s="68" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
     </row>
     <row r="18" spans="2:16">
       <c r="B18" s="48" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="D18" s="48" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="E18" s="48" t="s">
-        <v>431</v>
+        <v>424</v>
       </c>
       <c r="F18" s="48" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="G18" s="48" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="I18" s="65"/>
       <c r="J18" s="65" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K18" s="65"/>
       <c r="L18" s="65" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="N18" s="56"/>
       <c r="O18" s="56" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P18" s="68" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
     </row>
     <row r="19" spans="2:16">
       <c r="N19" s="56"/>
       <c r="O19" s="56"/>
       <c r="P19" s="68" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
     </row>
     <row r="20" spans="2:16">
       <c r="I20" s="60" t="s">
-        <v>463</v>
+        <v>456</v>
       </c>
       <c r="J20" s="60" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="K20" s="61" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="L20" s="62" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="N20" s="56"/>
       <c r="O20" s="54" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="P20" s="68" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
     </row>
     <row r="21" spans="2:16">
       <c r="I21" s="62"/>
       <c r="J21" s="61" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
       <c r="K21" s="61" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="L21" s="62" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="N21" s="56"/>
       <c r="O21" s="55" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
       <c r="P21" s="68" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="22" spans="2:16">
       <c r="I22" s="62"/>
       <c r="J22" s="62" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K22" s="61" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="L22" s="62" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="N22" s="56"/>
       <c r="O22" s="56" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P22" s="56"/>
     </row>
@@ -6613,10 +6940,10 @@
       <c r="I23" s="62"/>
       <c r="J23" s="62"/>
       <c r="K23" s="61" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="L23" s="62" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="N23" s="56"/>
       <c r="O23" s="56"/>
@@ -6625,174 +6952,174 @@
     <row r="24" spans="2:16">
       <c r="I24" s="62"/>
       <c r="J24" s="60" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="K24" s="61" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="L24" s="62" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="N24" s="56"/>
       <c r="O24" s="54" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="P24" s="56"/>
     </row>
     <row r="25" spans="2:16">
       <c r="I25" s="62"/>
       <c r="J25" s="61" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="K25" s="62"/>
       <c r="L25" s="62" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="N25" s="56"/>
       <c r="O25" s="55" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
       <c r="P25" s="56"/>
     </row>
     <row r="26" spans="2:16">
       <c r="I26" s="62"/>
       <c r="J26" s="62" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K26" s="62"/>
       <c r="L26" s="62" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="N26" s="56"/>
       <c r="O26" s="56" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P26" s="56"/>
     </row>
     <row r="28" spans="2:16">
       <c r="I28" s="57" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="J28" s="57" t="s">
+        <v>447</v>
+      </c>
+      <c r="K28" s="58" t="s">
+        <v>486</v>
+      </c>
+      <c r="L28" s="58" t="s">
+        <v>510</v>
+      </c>
+      <c r="N28" s="63" t="s">
+        <v>474</v>
+      </c>
+      <c r="O28" s="63" t="s">
         <v>454</v>
       </c>
-      <c r="K28" s="58" t="s">
-        <v>493</v>
-      </c>
-      <c r="L28" s="58" t="s">
-        <v>517</v>
-      </c>
-      <c r="N28" s="63" t="s">
-        <v>481</v>
-      </c>
-      <c r="O28" s="63" t="s">
-        <v>461</v>
-      </c>
       <c r="P28" s="65" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
     </row>
     <row r="29" spans="2:16">
       <c r="I29" s="59"/>
       <c r="J29" s="58" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="K29" s="58" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="L29" s="58" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="N29" s="65"/>
       <c r="O29" s="64" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="P29" s="65" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
     </row>
     <row r="30" spans="2:16">
       <c r="I30" s="59"/>
       <c r="J30" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K30" s="58" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="L30" s="58" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="N30" s="65"/>
       <c r="O30" s="65" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P30" s="65" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="31" spans="2:16">
       <c r="I31" s="59"/>
       <c r="J31" s="59"/>
       <c r="K31" s="58" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="L31" s="58" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="N31" s="65"/>
       <c r="O31" s="65"/>
       <c r="P31" s="65" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
     </row>
     <row r="32" spans="2:16">
       <c r="I32" s="59"/>
       <c r="J32" s="57" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="K32" s="58" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="L32" s="58" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="N32" s="65"/>
       <c r="O32" s="63" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
       <c r="P32" s="65" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33" spans="9:16">
       <c r="I33" s="59"/>
       <c r="J33" s="58" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="K33" s="59"/>
       <c r="L33" s="58" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="N33" s="65"/>
       <c r="O33" s="64" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="P33" s="65" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="34" spans="9:16">
       <c r="I34" s="59"/>
       <c r="J34" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K34" s="58"/>
       <c r="L34" s="58" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="N34" s="65"/>
       <c r="O34" s="65" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P34" s="65"/>
     </row>
@@ -6808,39 +7135,39 @@
     <row r="36" spans="9:16">
       <c r="I36" s="59"/>
       <c r="J36" s="57" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="K36" s="59"/>
       <c r="L36" s="59"/>
       <c r="N36" s="65"/>
       <c r="O36" s="63" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="P36" s="65"/>
     </row>
     <row r="37" spans="9:16">
       <c r="I37" s="59"/>
       <c r="J37" s="58" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="K37" s="59"/>
       <c r="L37" s="59"/>
       <c r="N37" s="65"/>
       <c r="O37" s="64" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="P37" s="65"/>
     </row>
     <row r="38" spans="9:16">
       <c r="I38" s="59"/>
       <c r="J38" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K38" s="58"/>
       <c r="L38" s="58"/>
       <c r="N38" s="65"/>
       <c r="O38" s="65" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P38" s="65"/>
     </row>
@@ -6853,55 +7180,55 @@
         <v>99</v>
       </c>
       <c r="J40" s="69" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="K40" s="52"/>
       <c r="L40" s="52"/>
       <c r="N40" s="57" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
       <c r="O40" s="57" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="P40" s="59" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
     </row>
     <row r="41" spans="9:16">
       <c r="I41" s="70"/>
       <c r="J41" s="71" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="K41" s="52"/>
       <c r="L41" s="52"/>
       <c r="N41" s="59"/>
       <c r="O41" s="58" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="P41" s="59" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
     </row>
     <row r="42" spans="9:16">
       <c r="I42" s="70"/>
       <c r="J42" s="70" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K42" s="53"/>
       <c r="L42" s="53"/>
       <c r="N42" s="59"/>
       <c r="O42" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P42" s="59" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
     </row>
     <row r="43" spans="9:16">
       <c r="N43" s="59"/>
       <c r="O43" s="59"/>
       <c r="P43" s="59" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
     </row>
     <row r="44" spans="9:16">
@@ -6909,45 +7236,45 @@
         <v>101</v>
       </c>
       <c r="J44" s="66" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="K44" s="55"/>
       <c r="L44" s="55" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="N44" s="59"/>
       <c r="O44" s="57" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="P44" s="59" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
     </row>
     <row r="45" spans="9:16">
       <c r="I45" s="68"/>
       <c r="J45" s="67" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="K45" s="55"/>
       <c r="L45" s="55"/>
       <c r="N45" s="59"/>
       <c r="O45" s="58" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
       <c r="P45" s="59" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
     </row>
     <row r="46" spans="9:16">
       <c r="I46" s="68"/>
       <c r="J46" s="68" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="K46" s="56"/>
       <c r="L46" s="56"/>
       <c r="N46" s="59"/>
       <c r="O46" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P46" s="59"/>
     </row>
@@ -6959,21 +7286,21 @@
     <row r="48" spans="9:16">
       <c r="N48" s="59"/>
       <c r="O48" s="57" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="P48" s="59"/>
     </row>
     <row r="49" spans="14:16">
       <c r="N49" s="59"/>
       <c r="O49" s="58" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="P49" s="59"/>
     </row>
     <row r="50" spans="14:16">
       <c r="N50" s="59"/>
       <c r="O50" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P50" s="59"/>
     </row>
@@ -6985,21 +7312,21 @@
     <row r="52" spans="14:16">
       <c r="N52" s="59"/>
       <c r="O52" s="57" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="P52" s="59"/>
     </row>
     <row r="53" spans="14:16">
       <c r="N53" s="59"/>
       <c r="O53" s="58" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="P53" s="59"/>
     </row>
     <row r="54" spans="14:16">
       <c r="N54" s="59"/>
       <c r="O54" s="59" t="s">
-        <v>456</v>
+        <v>449</v>
       </c>
       <c r="P54" s="59"/>
     </row>
@@ -7007,4 +7334,593 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B28EEAB-9943-4AF3-851F-40A6A33B4FB7}">
+  <dimension ref="B2:D71"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="51.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" s="9" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="15.75" thickBot="1">
+      <c r="C3" s="72" t="s">
+        <v>445</v>
+      </c>
+      <c r="D3" s="72" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="15.75" thickTop="1">
+      <c r="C4" s="73" t="s">
+        <v>528</v>
+      </c>
+      <c r="D4" s="73" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="C6" s="33" t="s">
+        <v>452</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="C7" s="33"/>
+      <c r="D7" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="C8" s="33"/>
+      <c r="D8" s="33" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+    </row>
+    <row r="10" spans="2:4">
+      <c r="C10" s="33"/>
+      <c r="D10" s="33" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4">
+      <c r="C11" s="33"/>
+      <c r="D11" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="C13" s="33" t="s">
+        <v>456</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="C14" s="33"/>
+      <c r="D14" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="C15" s="33"/>
+      <c r="D15" s="33" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+    </row>
+    <row r="17" spans="3:4">
+      <c r="C17" s="33"/>
+      <c r="D17" s="33" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4">
+      <c r="C18" s="33"/>
+      <c r="D18" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4">
+      <c r="C20" s="33" t="s">
+        <v>459</v>
+      </c>
+      <c r="D20" s="33" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4">
+      <c r="C21" s="33"/>
+      <c r="D21" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4">
+      <c r="C22" s="33"/>
+      <c r="D22" s="33" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4">
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+    </row>
+    <row r="24" spans="3:4">
+      <c r="C24" s="33"/>
+      <c r="D24" s="33" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4">
+      <c r="C25" s="33"/>
+      <c r="D25" s="33" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4">
+      <c r="C27" s="74" t="s">
+        <v>464</v>
+      </c>
+      <c r="D27" s="74" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="28" spans="3:4">
+      <c r="C28" s="74"/>
+      <c r="D28" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="29" spans="3:4">
+      <c r="C29" s="74"/>
+      <c r="D29" s="74" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="30" spans="3:4">
+      <c r="C30" s="74"/>
+      <c r="D30" s="74"/>
+    </row>
+    <row r="31" spans="3:4">
+      <c r="C31" s="74"/>
+      <c r="D31" s="75" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="32" spans="3:4">
+      <c r="C32" s="74"/>
+      <c r="D32" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="33" spans="3:4">
+      <c r="C33" s="74"/>
+      <c r="D33" s="75" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="34" spans="3:4">
+      <c r="C34" s="74"/>
+      <c r="D34" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="35" spans="3:4">
+      <c r="C35" s="74"/>
+      <c r="D35" s="75" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4">
+      <c r="C36" s="74"/>
+      <c r="D36" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="38" spans="3:4">
+      <c r="C38" s="75" t="s">
+        <v>470</v>
+      </c>
+      <c r="D38" s="74" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="39" spans="3:4">
+      <c r="C39" s="74"/>
+      <c r="D39" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="40" spans="3:4">
+      <c r="C40" s="74"/>
+      <c r="D40" s="74" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="41" spans="3:4">
+      <c r="C41" s="74"/>
+      <c r="D41" s="74"/>
+    </row>
+    <row r="42" spans="3:4">
+      <c r="C42" s="74"/>
+      <c r="D42" s="75" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="43" spans="3:4">
+      <c r="C43" s="74"/>
+      <c r="D43" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="44" spans="3:4">
+      <c r="C44" s="74"/>
+      <c r="D44" s="75" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="45" spans="3:4">
+      <c r="C45" s="74"/>
+      <c r="D45" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="46" spans="3:4">
+      <c r="C46" s="74"/>
+      <c r="D46" s="75" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="47" spans="3:4">
+      <c r="C47" s="74"/>
+      <c r="D47" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4">
+      <c r="C49" s="75" t="s">
+        <v>535</v>
+      </c>
+      <c r="D49" s="74" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="50" spans="3:4">
+      <c r="C50" s="74"/>
+      <c r="D50" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="51" spans="3:4">
+      <c r="C51" s="74"/>
+      <c r="D51" s="74" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="52" spans="3:4">
+      <c r="C52" s="74"/>
+      <c r="D52" s="74"/>
+    </row>
+    <row r="53" spans="3:4">
+      <c r="C53" s="74"/>
+      <c r="D53" s="75" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="54" spans="3:4">
+      <c r="C54" s="74"/>
+      <c r="D54" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="55" spans="3:4">
+      <c r="C55" s="74"/>
+      <c r="D55" s="75" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="56" spans="3:4">
+      <c r="C56" s="74"/>
+      <c r="D56" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="57" spans="3:4">
+      <c r="C57" s="74"/>
+      <c r="D57" s="75" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="58" spans="3:4">
+      <c r="C58" s="74"/>
+      <c r="D58" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="60" spans="3:4">
+      <c r="C60" s="75" t="s">
+        <v>479</v>
+      </c>
+      <c r="D60" s="74" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="61" spans="3:4">
+      <c r="C61" s="74"/>
+      <c r="D61" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="62" spans="3:4">
+      <c r="C62" s="74"/>
+      <c r="D62" s="74" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="63" spans="3:4">
+      <c r="C63" s="74"/>
+      <c r="D63" s="74"/>
+    </row>
+    <row r="64" spans="3:4">
+      <c r="C64" s="74"/>
+      <c r="D64" s="75" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="65" spans="3:4">
+      <c r="C65" s="74"/>
+      <c r="D65" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="66" spans="3:4">
+      <c r="C66" s="74"/>
+      <c r="D66" s="75" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="67" spans="3:4">
+      <c r="C67" s="74"/>
+      <c r="D67" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4">
+      <c r="C68" s="74"/>
+      <c r="D68" s="75" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="69" spans="3:4">
+      <c r="C69" s="74"/>
+      <c r="D69" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="70" spans="3:4">
+      <c r="C70" s="74"/>
+      <c r="D70" s="75" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="71" spans="3:4">
+      <c r="C71" s="74"/>
+      <c r="D71" s="74" t="s">
+        <v>530</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA218E61-637F-4B28-82C2-B126E3915C36}">
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" customWidth="1"/>
+    <col min="7" max="7" width="34.5703125" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15.75">
+      <c r="A1" t="s">
+        <v>548</v>
+      </c>
+      <c r="C1" s="76" t="s">
+        <v>536</v>
+      </c>
+      <c r="E1" s="77" t="s">
+        <v>540</v>
+      </c>
+      <c r="G1" t="s">
+        <v>550</v>
+      </c>
+      <c r="H1" t="s">
+        <v>445</v>
+      </c>
+      <c r="I1" t="s">
+        <v>551</v>
+      </c>
+      <c r="J1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C2" t="s">
+        <v>537</v>
+      </c>
+      <c r="E2" t="s">
+        <v>537</v>
+      </c>
+      <c r="H2" t="s">
+        <v>446</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="C3" t="s">
+        <v>533</v>
+      </c>
+      <c r="E3" t="s">
+        <v>533</v>
+      </c>
+      <c r="H3" t="s">
+        <v>446</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="C4" t="s">
+        <v>538</v>
+      </c>
+      <c r="E4" t="s">
+        <v>538</v>
+      </c>
+      <c r="H4" t="s">
+        <v>446</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="C5" t="s">
+        <v>539</v>
+      </c>
+      <c r="E5" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="C6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" t="s">
+        <v>172</v>
+      </c>
+      <c r="H6" t="s">
+        <v>450</v>
+      </c>
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="H7" t="s">
+        <v>450</v>
+      </c>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="C8" t="s">
+        <v>542</v>
+      </c>
+      <c r="E8" t="s">
+        <v>542</v>
+      </c>
+      <c r="H8" t="s">
+        <v>450</v>
+      </c>
+      <c r="I8" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="C9" t="s">
+        <v>543</v>
+      </c>
+      <c r="E9" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="C10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="C12" t="s">
+        <v>545</v>
+      </c>
+      <c r="E12" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="C13" t="s">
+        <v>546</v>
+      </c>
+      <c r="E13" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="C14" t="s">
+        <v>172</v>
+      </c>
+      <c r="E14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>